<commit_message>
updated matlab + Bode plotting
</commit_message>
<xml_diff>
--- a/Sims_and_Design/Pi Filter/PI Filter Values (RM_Electrical '26).xlsx
+++ b/Sims_and_Design/Pi Filter/PI Filter Values (RM_Electrical '26).xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\rm_electrical-supercap_v2\Sims_and_Design\Pi_filter_components\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\rm_electrical-supercap_v2\Sims_and_Design\Pi filter\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{C816BF5E-08B2-483B-B626-90B9C1F173A9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3EFCDB84-AE40-4CAB-8726-EE9B84961CCC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="3036" yWindow="3036" windowWidth="17280" windowHeight="9420" xr2:uid="{97A5CBE5-78E5-4C97-9F49-4F4237CD609D}"/>
   </bookViews>
@@ -50,9 +50,6 @@
     <t>a</t>
   </si>
   <si>
-    <t>L (mH)</t>
-  </si>
-  <si>
     <t>C (uF)</t>
   </si>
   <si>
@@ -63,6 +60,9 @@
   </si>
   <si>
     <t>1/(RC)</t>
+  </si>
+  <si>
+    <t>L (uH)</t>
   </si>
 </sst>
 </file>
@@ -434,7 +434,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2B73734A-272B-4037-BDFB-CE6B99C80540}">
-  <dimension ref="A1:K13"/>
+  <dimension ref="A1:K15"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="11" bestFit="1" customWidth="1"/>
@@ -454,19 +454,19 @@
         <v>3</v>
       </c>
       <c r="F1" t="s">
+        <v>8</v>
+      </c>
+      <c r="G1" t="s">
         <v>4</v>
       </c>
-      <c r="G1" t="s">
+      <c r="H1" t="s">
         <v>5</v>
       </c>
-      <c r="H1" t="s">
+      <c r="I1" t="s">
         <v>6</v>
       </c>
-      <c r="I1" t="s">
+      <c r="K1" t="s">
         <v>7</v>
-      </c>
-      <c r="K1" t="s">
-        <v>8</v>
       </c>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.3">
@@ -487,8 +487,8 @@
         <v>48780443.133604266</v>
       </c>
       <c r="F2">
-        <f>A2*1000</f>
-        <v>2.7E-2</v>
+        <f>A2*1000000</f>
+        <v>27</v>
       </c>
       <c r="G2">
         <v>10.07</v>
@@ -516,30 +516,30 @@
         <v>1.0439999999999998E-5</v>
       </c>
       <c r="C3">
-        <f t="shared" ref="C3:C13" si="2">A3*(24*3.1415+D3)</f>
+        <f t="shared" ref="C3:C15" si="2">A3*(24*3.1415+D3)</f>
         <v>1270.3961624731937</v>
       </c>
       <c r="D3">
-        <f t="shared" ref="D3:D13" si="3">1/(B3*A3*24*3.141592)</f>
+        <f t="shared" ref="D3:D15" si="3">1/(B3*A3*24*3.141592)</f>
         <v>47051634.325229399</v>
       </c>
       <c r="F3">
-        <f t="shared" ref="F3:F13" si="4">A3*1000</f>
-        <v>2.7E-2</v>
+        <f t="shared" ref="F3:F15" si="4">A3*1000000</f>
+        <v>27</v>
       </c>
       <c r="G3">
         <v>10.44</v>
       </c>
       <c r="H3">
-        <f t="shared" ref="H3:H13" si="5">C3/1000</f>
+        <f t="shared" ref="H3:H15" si="5">C3/1000</f>
         <v>1.2703961624731936</v>
       </c>
       <c r="I3">
-        <f t="shared" ref="I3:I13" si="6">D3/(2*3.1415)</f>
+        <f t="shared" ref="I3:I15" si="6">D3/(2*3.1415)</f>
         <v>7488721.0449195281</v>
       </c>
       <c r="K3">
-        <f t="shared" ref="K3:K13" si="7">1/(C3*B3)</f>
+        <f t="shared" ref="K3:K15" si="7">1/(C3*B3)</f>
         <v>75.398087181366137</v>
       </c>
     </row>
@@ -562,7 +562,7 @@
       </c>
       <c r="F4">
         <f t="shared" si="4"/>
-        <v>2.7E-2</v>
+        <v>27</v>
       </c>
       <c r="G4">
         <v>10.66</v>
@@ -599,7 +599,7 @@
       </c>
       <c r="F5">
         <f t="shared" si="4"/>
-        <v>2.7E-2</v>
+        <v>27</v>
       </c>
       <c r="G5">
         <v>10.88</v>
@@ -636,7 +636,7 @@
       </c>
       <c r="F6">
         <f t="shared" si="4"/>
-        <v>2.7E-2</v>
+        <v>27</v>
       </c>
       <c r="G6">
         <v>11.08</v>
@@ -673,7 +673,7 @@
       </c>
       <c r="F7">
         <f t="shared" si="4"/>
-        <v>2.7E-2</v>
+        <v>27</v>
       </c>
       <c r="G7">
         <v>11.09</v>
@@ -710,7 +710,7 @@
       </c>
       <c r="F8">
         <f t="shared" si="4"/>
-        <v>2.7E-2</v>
+        <v>27</v>
       </c>
       <c r="G8">
         <v>11.97</v>
@@ -747,7 +747,7 @@
       </c>
       <c r="F9">
         <f t="shared" si="4"/>
-        <v>2.7E-2</v>
+        <v>27</v>
       </c>
       <c r="G9">
         <v>12.48</v>
@@ -784,7 +784,7 @@
       </c>
       <c r="F10">
         <f t="shared" si="4"/>
-        <v>2.7E-2</v>
+        <v>27</v>
       </c>
       <c r="G10">
         <v>12.64</v>
@@ -821,7 +821,7 @@
       </c>
       <c r="F11">
         <f t="shared" si="4"/>
-        <v>2.7E-2</v>
+        <v>27</v>
       </c>
       <c r="G11">
         <v>12.67</v>
@@ -858,7 +858,7 @@
       </c>
       <c r="F12">
         <f t="shared" si="4"/>
-        <v>2.7E-2</v>
+        <v>27</v>
       </c>
       <c r="G12">
         <v>12.71</v>
@@ -895,7 +895,7 @@
       </c>
       <c r="F13">
         <f t="shared" si="4"/>
-        <v>2.7E-2</v>
+        <v>27</v>
       </c>
       <c r="G13">
         <v>12.88</v>
@@ -911,6 +911,78 @@
       <c r="K13">
         <f t="shared" si="7"/>
         <v>75.398058944116698</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A14">
+        <v>2.6999999999999999E-5</v>
+      </c>
+      <c r="B14">
+        <v>1.1E-5</v>
+      </c>
+      <c r="C14">
+        <f t="shared" si="2"/>
+        <v>1205.7215523825148</v>
+      </c>
+      <c r="D14">
+        <f t="shared" si="3"/>
+        <v>44656278.395944998</v>
+      </c>
+      <c r="F14">
+        <f t="shared" si="4"/>
+        <v>27</v>
+      </c>
+      <c r="G14">
+        <f>B14*1000000</f>
+        <v>11</v>
+      </c>
+      <c r="H14">
+        <f t="shared" si="5"/>
+        <v>1.2057215523825149</v>
+      </c>
+      <c r="I14">
+        <f t="shared" si="6"/>
+        <v>7107477.0644508982</v>
+      </c>
+      <c r="K14">
+        <f t="shared" si="7"/>
+        <v>75.398080700684062</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A15">
+        <v>2.6999999999999999E-5</v>
+      </c>
+      <c r="B15">
+        <v>1.2E-5</v>
+      </c>
+      <c r="C15">
+        <f t="shared" si="2"/>
+        <v>1105.2449259916384</v>
+      </c>
+      <c r="D15">
+        <f t="shared" si="3"/>
+        <v>40934921.862949573</v>
+      </c>
+      <c r="F15">
+        <f t="shared" si="4"/>
+        <v>27</v>
+      </c>
+      <c r="G15">
+        <f>B15*1000000</f>
+        <v>12</v>
+      </c>
+      <c r="H15">
+        <f t="shared" si="5"/>
+        <v>1.1052449259916384</v>
+      </c>
+      <c r="I15">
+        <f t="shared" si="6"/>
+        <v>6515187.3090799889</v>
+      </c>
+      <c r="K15">
+        <f t="shared" si="7"/>
+        <v>75.398069128040291</v>
       </c>
     </row>
   </sheetData>
@@ -1088,20 +1160,20 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_activity xmlns="edb1d2cc-d638-4107-bb2a-ead292282bd5" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
   <Edit>DocumentLibraryForm</Edit>
   <New>DocumentLibraryForm</New>
 </FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_activity xmlns="edb1d2cc-d638-4107-bb2a-ead292282bd5" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1123,6 +1195,14 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9DAC92D3-8B89-4153-BE4C-4D4D28F4CEE5}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CCD3BA36-27B7-4BA4-ADB4-FAF30231D7D8}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
@@ -1136,12 +1216,4 @@
     <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9DAC92D3-8B89-4153-BE4C-4D4D28F4CEE5}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>